<commit_message>
fix: Restore full 453-key TG matrix
</commit_message>
<xml_diff>
--- a/data_processing/Tesouro Gerencial Matriz.xlsx
+++ b/data_processing/Tesouro Gerencial Matriz.xlsx
@@ -4672,10 +4672,10 @@
         <v>39628.93</v>
       </c>
       <c r="I87" s="1">
-        <v>5954.2</v>
+        <v>0</v>
       </c>
       <c r="J87" s="1">
-        <v>33674.73</v>
+        <v>39628.93</v>
       </c>
       <c r="K87" s="1">
         <v>79257.86</v>
@@ -4736,10 +4736,10 @@
         <v>26355.84</v>
       </c>
       <c r="I89" s="1">
-        <v>5053.47</v>
+        <v>715.6</v>
       </c>
       <c r="J89" s="1">
-        <v>21302.37</v>
+        <v>25640.24</v>
       </c>
       <c r="K89" s="1">
         <v>53078.57</v>
@@ -4771,10 +4771,10 @@
         <v>1000</v>
       </c>
       <c r="I90" s="1">
-        <v>234.43</v>
+        <v>74.88</v>
       </c>
       <c r="J90" s="1">
-        <v>765.57</v>
+        <v>925.12</v>
       </c>
       <c r="K90" s="1">
         <v>2000</v>
@@ -5172,13 +5172,13 @@
         <v>16</v>
       </c>
       <c r="G103" s="1">
-        <v>706568.61</v>
+        <v>712568.61</v>
       </c>
       <c r="H103"/>
       <c r="I103"/>
       <c r="J103"/>
       <c r="K103" s="1">
-        <v>706568.61</v>
+        <v>712568.61</v>
       </c>
     </row>
     <row r="104">
@@ -5503,13 +5503,13 @@
         <v>16</v>
       </c>
       <c r="G114" s="1">
-        <v>221227.55</v>
+        <v>221057.55</v>
       </c>
       <c r="H114"/>
       <c r="I114"/>
       <c r="J114"/>
       <c r="K114" s="1">
-        <v>221227.55</v>
+        <v>221057.55</v>
       </c>
     </row>
     <row r="115">
@@ -5672,7 +5672,7 @@
         <v>63</v>
       </c>
       <c r="G119" s="1">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="H119" s="1">
         <v>2466.7</v>
@@ -5684,7 +5684,7 @@
         <v>2466.7</v>
       </c>
       <c r="K119" s="1">
-        <v>4933.4</v>
+        <v>5103.4</v>
       </c>
     </row>
     <row r="120">
@@ -8904,13 +8904,17 @@
         <v>47</v>
       </c>
       <c r="G217" s="1">
+        <v>0</v>
+      </c>
+      <c r="H217" s="1">
         <v>5320</v>
       </c>
-      <c r="H217"/>
-      <c r="I217"/>
+      <c r="I217" s="1">
+        <v>5320</v>
+      </c>
       <c r="J217"/>
       <c r="K217" s="1">
-        <v>5320</v>
+        <v>10640</v>
       </c>
     </row>
     <row r="218">
@@ -8933,13 +8937,17 @@
         <v>49</v>
       </c>
       <c r="G218" s="1">
+        <v>0</v>
+      </c>
+      <c r="H218" s="1">
         <v>12500</v>
       </c>
-      <c r="H218"/>
-      <c r="I218"/>
+      <c r="I218" s="1">
+        <v>12500</v>
+      </c>
       <c r="J218"/>
       <c r="K218" s="1">
-        <v>12500</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="219">
@@ -8962,13 +8970,17 @@
         <v>27</v>
       </c>
       <c r="G219" s="1">
+        <v>0</v>
+      </c>
+      <c r="H219" s="1">
         <v>13110</v>
       </c>
-      <c r="H219"/>
-      <c r="I219"/>
+      <c r="I219" s="1">
+        <v>13110</v>
+      </c>
       <c r="J219"/>
       <c r="K219" s="1">
-        <v>13110</v>
+        <v>26220</v>
       </c>
     </row>
     <row r="220">
@@ -9067,10 +9079,10 @@
         <v>50860</v>
       </c>
       <c r="I222" s="1">
-        <v>0</v>
+        <v>800</v>
       </c>
       <c r="J222" s="1">
-        <v>50860</v>
+        <v>50060</v>
       </c>
       <c r="K222" s="1">
         <v>101720</v>
@@ -10051,10 +10063,10 @@
         <v>1670200</v>
       </c>
       <c r="I252" s="1">
-        <v>209300</v>
+        <v>210700</v>
       </c>
       <c r="J252" s="1">
-        <v>1460900</v>
+        <v>1459500</v>
       </c>
       <c r="K252" s="1">
         <v>3340400</v>
@@ -10653,10 +10665,10 @@
         <v>4208071.2</v>
       </c>
       <c r="I270" s="1">
-        <v>1590882.2</v>
+        <v>1558731.94</v>
       </c>
       <c r="J270" s="1">
-        <v>2617189</v>
+        <v>2649339.26</v>
       </c>
       <c r="K270" s="1">
         <v>8419936</v>
@@ -11026,10 +11038,10 @@
         <v>468161.73</v>
       </c>
       <c r="I281" s="1">
-        <v>245754.47</v>
+        <v>245370.55</v>
       </c>
       <c r="J281" s="1">
-        <v>222407.26</v>
+        <v>222791.18</v>
       </c>
       <c r="K281" s="1">
         <v>936323.46</v>
@@ -11744,13 +11756,13 @@
         <v>16</v>
       </c>
       <c r="G303" s="1">
-        <v>527174.15</v>
+        <v>524174.15</v>
       </c>
       <c r="H303"/>
       <c r="I303"/>
       <c r="J303"/>
       <c r="K303" s="1">
-        <v>527174.15</v>
+        <v>524174.15</v>
       </c>
     </row>
     <row r="304">
@@ -11808,7 +11820,7 @@
         <v>49</v>
       </c>
       <c r="G305" s="1">
-        <v>31280</v>
+        <v>34280</v>
       </c>
       <c r="H305" s="1">
         <v>103142.51</v>
@@ -11820,7 +11832,7 @@
         <v>102342.51</v>
       </c>
       <c r="K305" s="1">
-        <v>237565.02</v>
+        <v>240565.02</v>
       </c>
     </row>
     <row r="306">
@@ -12070,13 +12082,13 @@
         <v>16</v>
       </c>
       <c r="G313" s="1">
-        <v>459132.26</v>
+        <v>456132.26</v>
       </c>
       <c r="H313"/>
       <c r="I313"/>
       <c r="J313"/>
       <c r="K313" s="1">
-        <v>459132.26</v>
+        <v>456132.26</v>
       </c>
     </row>
     <row r="314">
@@ -12099,7 +12111,7 @@
         <v>47</v>
       </c>
       <c r="G314" s="1">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="H314" s="1">
         <v>15998</v>
@@ -12111,7 +12123,7 @@
         <v>15593.92</v>
       </c>
       <c r="K314" s="1">
-        <v>31996</v>
+        <v>32996</v>
       </c>
     </row>
     <row r="315">
@@ -12239,7 +12251,7 @@
         <v>53</v>
       </c>
       <c r="G318" s="1">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="H318" s="1">
         <v>12000</v>
@@ -12251,7 +12263,7 @@
         <v>11323.2</v>
       </c>
       <c r="K318" s="1">
-        <v>24000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="319">
@@ -13159,10 +13171,10 @@
         <v>18000</v>
       </c>
       <c r="I346" s="1">
-        <v>13800</v>
+        <v>11400</v>
       </c>
       <c r="J346" s="1">
-        <v>4200</v>
+        <v>6600</v>
       </c>
       <c r="K346" s="1">
         <v>36000</v>
@@ -13415,13 +13427,13 @@
         <v>16</v>
       </c>
       <c r="G354" s="1">
-        <v>204729.82</v>
+        <v>196729.82</v>
       </c>
       <c r="H354"/>
       <c r="I354"/>
       <c r="J354"/>
       <c r="K354" s="1">
-        <v>204729.82</v>
+        <v>196729.82</v>
       </c>
     </row>
     <row r="355">
@@ -13444,7 +13456,7 @@
         <v>47</v>
       </c>
       <c r="G355" s="1">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="H355" s="1">
         <v>50000</v>
@@ -13456,7 +13468,7 @@
         <v>39906.06</v>
       </c>
       <c r="K355" s="1">
-        <v>100000</v>
+        <v>108000</v>
       </c>
     </row>
     <row r="356">
@@ -14044,10 +14056,10 @@
         <v>58400</v>
       </c>
       <c r="I373" s="1">
-        <v>36500</v>
+        <v>29200</v>
       </c>
       <c r="J373" s="1">
-        <v>21900</v>
+        <v>29200</v>
       </c>
       <c r="K373" s="1">
         <v>116800</v>
@@ -14456,9 +14468,11 @@
         <v>172269.71</v>
       </c>
       <c r="I385" s="1">
-        <v>172269.71</v>
-      </c>
-      <c r="J385"/>
+        <v>1014.23</v>
+      </c>
+      <c r="J385" s="1">
+        <v>171255.48</v>
+      </c>
       <c r="K385" s="1">
         <v>344539.42</v>
       </c>
@@ -14838,17 +14852,17 @@
         <v>18</v>
       </c>
       <c r="G397" s="1">
-        <v>9100</v>
+        <v>100</v>
       </c>
       <c r="H397" s="1">
-        <v>22400</v>
+        <v>31400</v>
       </c>
       <c r="I397" s="1">
-        <v>22400</v>
+        <v>31400</v>
       </c>
       <c r="J397"/>
       <c r="K397" s="1">
-        <v>53900</v>
+        <v>62900</v>
       </c>
     </row>
     <row r="398">
@@ -15457,10 +15471,10 @@
         <v>10268.6</v>
       </c>
       <c r="I416" s="1">
-        <v>4418.6</v>
+        <v>2529</v>
       </c>
       <c r="J416" s="1">
-        <v>5850</v>
+        <v>7739.6</v>
       </c>
       <c r="K416" s="1">
         <v>20637.2</v>
@@ -16214,10 +16228,10 @@
         <v>20469.63</v>
       </c>
       <c r="I439" s="1">
-        <v>12434.32</v>
+        <v>3794.32</v>
       </c>
       <c r="J439" s="1">
-        <v>8035.31</v>
+        <v>16675.31</v>
       </c>
       <c r="K439" s="1">
         <v>40939.26</v>
@@ -16243,13 +16257,13 @@
         <v>16</v>
       </c>
       <c r="G440" s="1">
-        <v>10496</v>
+        <v>6075.84</v>
       </c>
       <c r="H440"/>
       <c r="I440"/>
       <c r="J440"/>
       <c r="K440" s="1">
-        <v>10496</v>
+        <v>6075.84</v>
       </c>
     </row>
     <row r="441">
@@ -16377,7 +16391,7 @@
         <v>27</v>
       </c>
       <c r="G444" s="1">
-        <v>0</v>
+        <v>4420.16</v>
       </c>
       <c r="H444" s="1">
         <v>11904</v>
@@ -16389,7 +16403,7 @@
         <v>11904</v>
       </c>
       <c r="K444" s="1">
-        <v>23808</v>
+        <v>28228.16</v>
       </c>
     </row>
     <row r="445">
@@ -17972,19 +17986,19 @@
         <v>18</v>
       </c>
       <c r="G493" s="1">
-        <v>50263.5</v>
+        <v>8.58</v>
       </c>
       <c r="H493" s="1">
-        <v>13491.42</v>
+        <v>63746.34</v>
       </c>
       <c r="I493" s="1">
-        <v>0</v>
+        <v>50254.92</v>
       </c>
       <c r="J493" s="1">
         <v>13491.42</v>
       </c>
       <c r="K493" s="1">
-        <v>77246.34</v>
+        <v>127501.26</v>
       </c>
     </row>
     <row r="494">
@@ -19277,13 +19291,13 @@
         <v>16</v>
       </c>
       <c r="G534" s="1">
-        <v>514841.02</v>
+        <v>500541.02</v>
       </c>
       <c r="H534"/>
       <c r="I534"/>
       <c r="J534"/>
       <c r="K534" s="1">
-        <v>514841.02</v>
+        <v>500541.02</v>
       </c>
     </row>
     <row r="535">
@@ -19341,7 +19355,7 @@
         <v>49</v>
       </c>
       <c r="G536" s="1">
-        <v>0</v>
+        <v>14300</v>
       </c>
       <c r="H536" s="1">
         <v>120065</v>
@@ -19353,7 +19367,7 @@
         <v>119790</v>
       </c>
       <c r="K536" s="1">
-        <v>240130</v>
+        <v>254430</v>
       </c>
     </row>
     <row r="537">
@@ -20353,10 +20367,10 @@
         <v>644677.6</v>
       </c>
       <c r="I566" s="1">
-        <v>111101.39</v>
+        <v>31918.96</v>
       </c>
       <c r="J566" s="1">
-        <v>533576.21</v>
+        <v>612758.64</v>
       </c>
       <c r="K566" s="1">
         <v>1294355.2</v>
@@ -20695,10 +20709,10 @@
         <v>180000</v>
       </c>
       <c r="I576" s="1">
-        <v>70764.7</v>
+        <v>70705.71</v>
       </c>
       <c r="J576" s="1">
-        <v>109235.3</v>
+        <v>109294.29</v>
       </c>
       <c r="K576" s="1">
         <v>440000</v>
@@ -21093,10 +21107,10 @@
         <v>352717.14</v>
       </c>
       <c r="I588" s="1">
-        <v>84404.21</v>
+        <v>83712.31</v>
       </c>
       <c r="J588" s="1">
-        <v>268312.93</v>
+        <v>269004.83</v>
       </c>
       <c r="K588" s="1">
         <v>705434.28</v>
@@ -21989,13 +22003,13 @@
         <v>16</v>
       </c>
       <c r="G616" s="1">
-        <v>31899.77</v>
+        <v>28199.77</v>
       </c>
       <c r="H616"/>
       <c r="I616"/>
       <c r="J616"/>
       <c r="K616" s="1">
-        <v>31899.77</v>
+        <v>28199.77</v>
       </c>
     </row>
     <row r="617">
@@ -22018,7 +22032,7 @@
         <v>47</v>
       </c>
       <c r="G617" s="1">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="H617" s="1">
         <v>6500</v>
@@ -22030,7 +22044,7 @@
         <v>5899.51</v>
       </c>
       <c r="K617" s="1">
-        <v>13000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="618">
@@ -22053,7 +22067,7 @@
         <v>53</v>
       </c>
       <c r="G618" s="1">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="H618" s="1">
         <v>5000</v>
@@ -22065,7 +22079,7 @@
         <v>3505.1</v>
       </c>
       <c r="K618" s="1">
-        <v>10000</v>
+        <v>10700</v>
       </c>
     </row>
     <row r="619">
@@ -22294,9 +22308,11 @@
         <v>13100</v>
       </c>
       <c r="I625" s="1">
-        <v>13100</v>
-      </c>
-      <c r="J625"/>
+        <v>6100</v>
+      </c>
+      <c r="J625" s="1">
+        <v>7000</v>
+      </c>
       <c r="K625" s="1">
         <v>26200</v>
       </c>
@@ -22676,19 +22692,19 @@
         <v>47</v>
       </c>
       <c r="G637" s="1">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="H637" s="1">
-        <v>62000</v>
+        <v>63000</v>
       </c>
       <c r="I637" s="1">
-        <v>5685.61</v>
+        <v>6685.61</v>
       </c>
       <c r="J637" s="1">
         <v>56314.39</v>
       </c>
       <c r="K637" s="1">
-        <v>125000</v>
+        <v>126000</v>
       </c>
     </row>
     <row r="638">
@@ -22810,19 +22826,19 @@
         <v>53</v>
       </c>
       <c r="G641" s="1">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="H641" s="1">
-        <v>38200</v>
+        <v>43200</v>
       </c>
       <c r="I641" s="1">
-        <v>11458.25</v>
+        <v>16458.25</v>
       </c>
       <c r="J641" s="1">
         <v>26741.75</v>
       </c>
       <c r="K641" s="1">
-        <v>81400</v>
+        <v>86400</v>
       </c>
     </row>
     <row r="642">
@@ -23175,13 +23191,13 @@
         <v>16</v>
       </c>
       <c r="G652" s="1">
-        <v>113096.73</v>
+        <v>82096.73</v>
       </c>
       <c r="H652"/>
       <c r="I652"/>
       <c r="J652"/>
       <c r="K652" s="1">
-        <v>113096.73</v>
+        <v>82096.73</v>
       </c>
     </row>
     <row r="653">
@@ -23204,7 +23220,7 @@
         <v>47</v>
       </c>
       <c r="G653" s="1">
-        <v>0</v>
+        <v>16000</v>
       </c>
       <c r="H653" s="1">
         <v>45867.5</v>
@@ -23216,7 +23232,7 @@
         <v>33760.96</v>
       </c>
       <c r="K653" s="1">
-        <v>91735</v>
+        <v>107735</v>
       </c>
     </row>
     <row r="654">
@@ -23342,7 +23358,7 @@
         <v>53</v>
       </c>
       <c r="G657" s="1">
-        <v>0</v>
+        <v>15000</v>
       </c>
       <c r="H657" s="1">
         <v>89900</v>
@@ -23354,7 +23370,7 @@
         <v>6514.94</v>
       </c>
       <c r="K657" s="1">
-        <v>179800</v>
+        <v>194800</v>
       </c>
     </row>
     <row r="658">
@@ -24418,13 +24434,13 @@
         <v>16</v>
       </c>
       <c r="G691" s="1">
-        <v>361914.82</v>
+        <v>326057.16</v>
       </c>
       <c r="H691"/>
       <c r="I691"/>
       <c r="J691"/>
       <c r="K691" s="1">
-        <v>361914.82</v>
+        <v>326057.16</v>
       </c>
     </row>
     <row r="692">
@@ -24517,7 +24533,7 @@
         <v>35</v>
       </c>
       <c r="G694" s="1">
-        <v>3E-02</v>
+        <v>35857.69</v>
       </c>
       <c r="H694" s="1">
         <v>198702.09</v>
@@ -24529,7 +24545,7 @@
         <v>192467.55</v>
       </c>
       <c r="K694" s="1">
-        <v>397404.21</v>
+        <v>433261.87</v>
       </c>
     </row>
     <row r="695">
@@ -27062,19 +27078,19 @@
         <v>47</v>
       </c>
       <c r="G773" s="1">
-        <v>0</v>
+        <v>18106.23</v>
       </c>
       <c r="H773" s="1">
-        <v>95000</v>
+        <v>76893.77</v>
       </c>
       <c r="I773" s="1">
-        <v>29468.09</v>
+        <v>11361.86</v>
       </c>
       <c r="J773" s="1">
         <v>65531.91</v>
       </c>
       <c r="K773" s="1">
-        <v>190000</v>
+        <v>171893.77</v>
       </c>
     </row>
     <row r="774">
@@ -27415,13 +27431,13 @@
         <v>16</v>
       </c>
       <c r="G784" s="1">
-        <v>426012.45</v>
+        <v>420012.45</v>
       </c>
       <c r="H784"/>
       <c r="I784"/>
       <c r="J784"/>
       <c r="K784" s="1">
-        <v>426012.45</v>
+        <v>420012.45</v>
       </c>
     </row>
     <row r="785">
@@ -27450,10 +27466,10 @@
         <v>25165</v>
       </c>
       <c r="I785" s="1">
-        <v>15125.83</v>
+        <v>14283.02</v>
       </c>
       <c r="J785" s="1">
-        <v>10039.17</v>
+        <v>10881.98</v>
       </c>
       <c r="K785" s="1">
         <v>50330</v>
@@ -30503,19 +30519,19 @@
         <v>51</v>
       </c>
       <c r="G880" s="1">
-        <v>5000.03</v>
+        <v>4963.03</v>
       </c>
       <c r="H880" s="1">
-        <v>197368.32</v>
+        <v>197405.32</v>
       </c>
       <c r="I880" s="1">
-        <v>104884.5</v>
+        <v>101257.8</v>
       </c>
       <c r="J880" s="1">
-        <v>92483.82</v>
+        <v>96147.52</v>
       </c>
       <c r="K880" s="1">
-        <v>399736.67</v>
+        <v>399773.67</v>
       </c>
     </row>
     <row r="881">
@@ -31464,10 +31480,10 @@
         <v>53111.48</v>
       </c>
       <c r="I909" s="1">
-        <v>10564.15</v>
+        <v>4709.97</v>
       </c>
       <c r="J909" s="1">
-        <v>42547.33</v>
+        <v>48401.51</v>
       </c>
       <c r="K909" s="1">
         <v>106222.96</v>
@@ -31528,19 +31544,19 @@
         <v>113</v>
       </c>
       <c r="G911" s="1">
-        <v>172370.22</v>
+        <v>0</v>
       </c>
       <c r="H911" s="1">
-        <v>814738.57</v>
+        <v>987108.79</v>
       </c>
       <c r="I911" s="1">
-        <v>73604.37</v>
+        <v>245974.59</v>
       </c>
       <c r="J911" s="1">
         <v>741134.2</v>
       </c>
       <c r="K911" s="1">
-        <v>1801847.36</v>
+        <v>1974217.58</v>
       </c>
     </row>
     <row r="912">
@@ -33451,19 +33467,19 @@
       <c r="E970" t="s"/>
       <c r="F970"/>
       <c r="G970" s="1">
-        <v>74158049.41</v>
+        <v>73907563.5</v>
       </c>
       <c r="H970" s="1">
-        <v>168378683.59</v>
+        <v>168629169.5</v>
       </c>
       <c r="I970" s="1">
-        <v>33221022.17</v>
+        <v>33141943.19</v>
       </c>
       <c r="J970" s="1">
-        <v>135157661.42</v>
+        <v>135487226.31</v>
       </c>
       <c r="K970" s="1">
-        <v>410915416.59</v>
+        <v>411165902.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>